<commit_message>
PF-1 fix 1.4 (F4, F3): perturb the copied sample figures; allow-list every text cell
scripts/build_templates.py: the five top-holding and Holdings_Detail tuples
(rating, sector, maturity, par, market value, % NAV) and the copied
aggregates (par, obligor, position and sector counts, WAR, WAS, YTM, WAL,
price, top-10, rating, sector and maturity bucket figures, Mandate free-row
dates and amounts) are new round illustrative figures. Kept: NAV, the five
design limits, C-01's 2.37 / 0.13 / Watch, Unrated 3.73 and CCC + Other +
Unrated = 7.36 (C-04, C-05), SECTOR's 4.57 and first-lien 99.39 (= 100 -
C-10's 0.61); buckets sum to 100.00. Template regenerated; byte stability
holds and the RV-1 template is unchanged.

The subset allow-list test is replaced by one that reads every text cell of
the committed template and compares it, both ways, with a literal list in
the test plus the headers and README lines.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/templates/portfolio.template.xlsx
+++ b/docs/templates/portfolio.template.xlsx
@@ -136,7 +136,7 @@
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-03-15 to 2027-03-15</t>
+          <t xml:space="preserve">2025-04-15 to 2027-04-15</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
@@ -158,7 +158,7 @@
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2038-03-15</t>
+          <t xml:space="preserve">2038-04-15</t>
         </is>
       </c>
     </row>
@@ -248,7 +248,7 @@
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">USD 50,000,000</t>
+          <t xml:space="preserve">USD 45,000,000</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
@@ -309,7 +309,7 @@
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">15 bps p.a. on collateral balance</t>
+          <t xml:space="preserve">20 bps p.a. on collateral balance</t>
         </is>
       </c>
     </row>
@@ -414,7 +414,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>634000000</v>
+        <v>635000000</v>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
@@ -434,7 +434,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>350</v>
+        <v>300</v>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
@@ -454,7 +454,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>383</v>
+        <v>320</v>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
@@ -494,11 +494,11 @@
         </is>
       </c>
       <c r="B7">
-        <v>14.3</v>
+        <v>14.0</v>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">rating notch (B1)</t>
+          <t xml:space="preserve">rating notch</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -514,7 +514,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>3.29</v>
+        <v>3.50</v>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
@@ -554,7 +554,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>4.82</v>
+        <v>4.50</v>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B11">
-        <v>99.578</v>
+        <v>99.50</v>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="B13">
-        <v>11.05</v>
+        <v>11.00</v>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
@@ -663,10 +663,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.32</v>
+        <v>0.50</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -676,10 +676,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>25.02</v>
+        <v>25.00</v>
       </c>
       <c r="C3">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4">
@@ -689,10 +689,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>67.30</v>
+        <v>67.14</v>
       </c>
       <c r="C4">
-        <v>259</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5">
@@ -702,10 +702,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>3.50</v>
+        <v>3.40</v>
       </c>
       <c r="C6">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -731,7 +731,7 @@
         <v>3.73</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -784,20 +784,20 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Care Facilities &amp; Services</t>
+          <t xml:space="preserve">Health Care Services</t>
         </is>
       </c>
       <c r="B2">
-        <v>7.16</v>
+        <v>7.00</v>
       </c>
       <c r="C2">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D2">
         <v>10.0</v>
       </c>
       <c r="E2">
-        <v>2.84</v>
+        <v>3.00</v>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
@@ -808,20 +808,20 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Commercial Support Services</t>
+          <t xml:space="preserve">Business Services</t>
         </is>
       </c>
       <c r="B3">
-        <v>6.74</v>
+        <v>6.50</v>
       </c>
       <c r="C3">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D3">
         <v>10.0</v>
       </c>
       <c r="E3">
-        <v>3.26</v>
+        <v>3.50</v>
       </c>
       <c r="F3" s="1" t="inlineStr">
         <is>
@@ -832,20 +832,20 @@
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insurance</t>
+          <t xml:space="preserve">Software</t>
         </is>
       </c>
       <c r="B4">
-        <v>5.63</v>
+        <v>5.75</v>
       </c>
       <c r="C4">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="D4">
         <v>10.0</v>
       </c>
       <c r="E4">
-        <v>4.37</v>
+        <v>4.25</v>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
@@ -856,20 +856,20 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Software</t>
+          <t xml:space="preserve">Chemicals</t>
         </is>
       </c>
       <c r="B5">
-        <v>5.31</v>
+        <v>5.25</v>
       </c>
       <c r="C5">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="D5">
         <v>10.0</v>
       </c>
       <c r="E5">
-        <v>4.69</v>
+        <v>4.75</v>
       </c>
       <c r="F5" s="1" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         <v>4.57</v>
       </c>
       <c r="C6">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>10.0</v>
@@ -961,7 +961,7 @@
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3 / B</t>
+          <t xml:space="preserve">B2 / B+</t>
         </is>
       </c>
     </row>
@@ -980,11 +980,11 @@
         </is>
       </c>
       <c r="D3">
-        <v>1.91</v>
+        <v>1.80</v>
       </c>
       <c r="E3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ba3 / BB-</t>
+          <t xml:space="preserve">Ba2 / BB</t>
         </is>
       </c>
     </row>
@@ -1003,11 +1003,11 @@
         </is>
       </c>
       <c r="D4">
-        <v>1.42</v>
+        <v>1.50</v>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2 / B</t>
+          <t xml:space="preserve">B3 / B-</t>
         </is>
       </c>
     </row>
@@ -1026,11 +1026,11 @@
         </is>
       </c>
       <c r="D5">
-        <v>0.96</v>
+        <v>1.10</v>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B1 / B+</t>
+          <t xml:space="preserve">B1 / B</t>
         </is>
       </c>
     </row>
@@ -1049,11 +1049,11 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.96</v>
+        <v>0.90</v>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2 / B+</t>
+          <t xml:space="preserve">Ba3 / BB-</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.15</v>
+        <v>0.50</v>
       </c>
     </row>
     <row r="3">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>3.78</v>
+        <v>4.00</v>
       </c>
     </row>
     <row r="4">
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>12.56</v>
+        <v>12.00</v>
       </c>
     </row>
     <row r="5">
@@ -1117,7 +1117,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>29.20</v>
+        <v>30.00</v>
       </c>
     </row>
     <row r="6">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>54.31</v>
+        <v>53.50</v>
       </c>
     </row>
   </sheetData>
@@ -1615,19 +1615,19 @@
         <v>15000000</v>
       </c>
       <c r="E2">
-        <v>14951250</v>
+        <v>14962500</v>
       </c>
       <c r="F2">
         <v>2.37</v>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B3 / B</t>
+          <t xml:space="preserve">B2 / B+</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insurance</t>
+          <t xml:space="preserve">Software</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2030-06-30</t>
+          <t xml:space="preserve">2030-09-30</t>
         </is>
       </c>
     </row>
@@ -1658,22 +1658,22 @@
         </is>
       </c>
       <c r="D3">
-        <v>12100000</v>
+        <v>11400000</v>
       </c>
       <c r="E3">
-        <v>12043500</v>
+        <v>11357000</v>
       </c>
       <c r="F3">
-        <v>1.91</v>
+        <v>1.80</v>
       </c>
       <c r="G3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ba3 / BB-</t>
+          <t xml:space="preserve">Ba2 / BB</t>
         </is>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aerospace &amp; Defense</t>
+          <t xml:space="preserve">Business Services</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2031-03-31</t>
+          <t xml:space="preserve">2031-06-30</t>
         </is>
       </c>
     </row>
@@ -1704,22 +1704,22 @@
         </is>
       </c>
       <c r="D4">
-        <v>9000000</v>
+        <v>9500000</v>
       </c>
       <c r="E4">
-        <v>8990625</v>
+        <v>9464000</v>
       </c>
       <c r="F4">
-        <v>1.42</v>
+        <v>1.50</v>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2 / B</t>
+          <t xml:space="preserve">B3 / B-</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment Content</t>
+          <t xml:space="preserve">Health Care Services</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="J4" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2029-12-31</t>
+          <t xml:space="preserve">2029-03-31</t>
         </is>
       </c>
     </row>
@@ -1750,22 +1750,22 @@
         </is>
       </c>
       <c r="D5">
-        <v>6100000</v>
+        <v>7000000</v>
       </c>
       <c r="E5">
-        <v>6031875</v>
+        <v>6940000</v>
       </c>
       <c r="F5">
-        <v>0.96</v>
+        <v>1.10</v>
       </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B1 / B+</t>
+          <t xml:space="preserve">B1 / B</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable &amp; Satellite</t>
+          <t xml:space="preserve">Chemicals</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="J5" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">2028-09-30</t>
+          <t xml:space="preserve">2028-12-31</t>
         </is>
       </c>
     </row>
@@ -1796,17 +1796,17 @@
         </is>
       </c>
       <c r="D6">
-        <v>6000000</v>
+        <v>5700000</v>
       </c>
       <c r="E6">
-        <v>6026250</v>
+        <v>5678400</v>
       </c>
       <c r="F6">
-        <v>0.96</v>
+        <v>0.90</v>
       </c>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">B2 / B+</t>
+          <t xml:space="preserve">Ba3 / BB-</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">

</xml_diff>